<commit_message>
Complete set of results and plots
</commit_message>
<xml_diff>
--- a/src/ereznic2/Results_main/hybrid_offgrid_results_summary.xlsx
+++ b/src/ereznic2/Results_main/hybrid_offgrid_results_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="25">
   <si>
     <t>2022</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>MN</t>
+  </si>
+  <si>
+    <t>Excess VRE capacity (%)</t>
   </si>
   <si>
     <t>Wind capacity (MW)</t>
@@ -457,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD47"/>
+  <dimension ref="A1:AD50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:30">
@@ -465,13 +468,13 @@
         <v>0</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:30">
@@ -555,73 +558,73 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>870</v>
+        <v>20</v>
       </c>
       <c r="C4">
-        <v>1002</v>
+        <v>10</v>
       </c>
       <c r="D4">
-        <v>838</v>
+        <v>10</v>
       </c>
       <c r="E4">
-        <v>1284</v>
+        <v>10</v>
       </c>
       <c r="F4">
-        <v>1248</v>
+        <v>10</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="J4">
-        <v>870</v>
+        <v>20</v>
       </c>
       <c r="K4">
-        <v>1002</v>
+        <v>10</v>
       </c>
       <c r="L4">
-        <v>838</v>
+        <v>10</v>
       </c>
       <c r="M4">
-        <v>1284</v>
+        <v>10</v>
       </c>
       <c r="N4">
-        <v>1248</v>
+        <v>10</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="R4">
-        <v>870</v>
+        <v>10</v>
       </c>
       <c r="S4">
-        <v>1002</v>
+        <v>10</v>
       </c>
       <c r="T4">
-        <v>838</v>
+        <v>10</v>
       </c>
       <c r="U4">
-        <v>1080</v>
+        <v>10</v>
       </c>
       <c r="V4">
-        <v>1248</v>
+        <v>10</v>
       </c>
       <c r="Y4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="Z4">
-        <v>870</v>
+        <v>20</v>
       </c>
       <c r="AA4">
-        <v>1002</v>
+        <v>10</v>
       </c>
       <c r="AB4">
-        <v>838</v>
+        <v>10</v>
       </c>
       <c r="AC4">
-        <v>882</v>
+        <v>10</v>
       </c>
       <c r="AD4">
-        <v>1248</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:30">
@@ -629,73 +632,73 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>800</v>
+        <v>822</v>
       </c>
       <c r="C5">
-        <v>100</v>
+        <v>888</v>
       </c>
       <c r="D5">
-        <v>700</v>
+        <v>722</v>
       </c>
       <c r="E5">
-        <v>300</v>
+        <v>1032</v>
       </c>
       <c r="F5">
-        <v>100</v>
+        <v>930</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J5">
-        <v>800</v>
+        <v>696</v>
       </c>
       <c r="K5">
-        <v>100</v>
+        <v>888</v>
       </c>
       <c r="L5">
-        <v>700</v>
+        <v>722</v>
       </c>
       <c r="M5">
-        <v>300</v>
+        <v>1032</v>
       </c>
       <c r="N5">
-        <v>100</v>
+        <v>930</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="R5">
-        <v>800</v>
+        <v>690</v>
       </c>
       <c r="S5">
-        <v>100</v>
+        <v>888</v>
       </c>
       <c r="T5">
-        <v>700</v>
+        <v>722</v>
       </c>
       <c r="U5">
-        <v>600</v>
+        <v>888</v>
       </c>
       <c r="V5">
-        <v>100</v>
+        <v>930</v>
       </c>
       <c r="Y5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="Z5">
-        <v>800</v>
+        <v>696</v>
       </c>
       <c r="AA5">
-        <v>100</v>
+        <v>756</v>
       </c>
       <c r="AB5">
-        <v>700</v>
+        <v>722</v>
       </c>
       <c r="AC5">
-        <v>900</v>
+        <v>888</v>
       </c>
       <c r="AD5">
-        <v>100</v>
+        <v>930</v>
       </c>
     </row>
     <row r="6" spans="1:30">
@@ -703,73 +706,73 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="T6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="V6">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="Y6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="Z6">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="AA6">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="AB6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="AC6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="AD6">
-        <v>0</v>
+        <v>800</v>
       </c>
     </row>
     <row r="7" spans="1:30">
@@ -777,73 +780,73 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="L7">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="M7">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="R7">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="S7">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="T7">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="U7">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="V7">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="Y7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="Z7">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="AA7">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="AB7">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="AC7">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="AD7">
-        <v>0</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:30">
@@ -851,73 +854,73 @@
         <v>11</v>
       </c>
       <c r="B8">
-        <v>1320</v>
+        <v>1</v>
       </c>
       <c r="C8">
-        <v>800</v>
+        <v>1</v>
       </c>
       <c r="D8">
-        <v>1240</v>
+        <v>1</v>
       </c>
       <c r="E8">
-        <v>1160</v>
+        <v>1</v>
       </c>
       <c r="F8">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J8">
-        <v>1320</v>
+        <v>1</v>
       </c>
       <c r="K8">
-        <v>800</v>
+        <v>1</v>
       </c>
       <c r="L8">
-        <v>1240</v>
+        <v>1</v>
       </c>
       <c r="M8">
-        <v>1160</v>
+        <v>1</v>
       </c>
       <c r="N8">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="R8">
-        <v>1320</v>
+        <v>1</v>
       </c>
       <c r="S8">
-        <v>800</v>
+        <v>1</v>
       </c>
       <c r="T8">
-        <v>1240</v>
+        <v>1</v>
       </c>
       <c r="U8">
-        <v>1280</v>
+        <v>1</v>
       </c>
       <c r="V8">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="Y8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="Z8">
-        <v>1320</v>
+        <v>1</v>
       </c>
       <c r="AA8">
-        <v>800</v>
+        <v>1</v>
       </c>
       <c r="AB8">
-        <v>1240</v>
+        <v>1</v>
       </c>
       <c r="AC8">
-        <v>1400</v>
+        <v>1</v>
       </c>
       <c r="AD8">
-        <v>1000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:30">
@@ -925,73 +928,73 @@
         <v>12</v>
       </c>
       <c r="B9">
-        <v>0.387</v>
+        <v>760</v>
       </c>
       <c r="C9">
-        <v>0.612</v>
+        <v>640</v>
       </c>
       <c r="D9">
-        <v>0.415</v>
+        <v>800</v>
       </c>
       <c r="E9">
-        <v>0.433</v>
+        <v>720</v>
       </c>
       <c r="F9">
-        <v>0.492</v>
+        <v>720</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>12</v>
       </c>
       <c r="J9">
-        <v>0.387</v>
+        <v>840</v>
       </c>
       <c r="K9">
-        <v>0.612</v>
+        <v>640</v>
       </c>
       <c r="L9">
-        <v>0.415</v>
+        <v>800</v>
       </c>
       <c r="M9">
-        <v>0.433</v>
+        <v>720</v>
       </c>
       <c r="N9">
-        <v>0.492</v>
+        <v>720</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R9">
-        <v>0.387</v>
+        <v>920</v>
       </c>
       <c r="S9">
-        <v>0.612</v>
+        <v>640</v>
       </c>
       <c r="T9">
-        <v>0.415</v>
+        <v>800</v>
       </c>
       <c r="U9">
-        <v>0.401</v>
+        <v>760</v>
       </c>
       <c r="V9">
-        <v>0.492</v>
+        <v>720</v>
       </c>
       <c r="Y9" s="2" t="s">
         <v>12</v>
       </c>
       <c r="Z9">
-        <v>0.387</v>
+        <v>840</v>
       </c>
       <c r="AA9">
-        <v>0.612</v>
+        <v>680</v>
       </c>
       <c r="AB9">
-        <v>0.415</v>
+        <v>800</v>
       </c>
       <c r="AC9">
-        <v>0.365</v>
+        <v>760</v>
       </c>
       <c r="AD9">
-        <v>0.492</v>
+        <v>720</v>
       </c>
     </row>
     <row r="10" spans="1:30">
@@ -999,73 +1002,73 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <v>4.37</v>
+        <v>0.628</v>
       </c>
       <c r="C10">
-        <v>5.25</v>
+        <v>0.729</v>
       </c>
       <c r="D10">
-        <v>4.69</v>
+        <v>0.602</v>
       </c>
       <c r="E10">
-        <v>4.09</v>
+        <v>0.65</v>
       </c>
       <c r="F10">
-        <v>4.5</v>
+        <v>0.662</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>13</v>
       </c>
       <c r="J10">
-        <v>4.37</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="K10">
-        <v>5.25</v>
+        <v>0.729</v>
       </c>
       <c r="L10">
-        <v>4.69</v>
+        <v>0.602</v>
       </c>
       <c r="M10">
-        <v>4.09</v>
+        <v>0.65</v>
       </c>
       <c r="N10">
-        <v>4.5</v>
+        <v>0.662</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>13</v>
       </c>
       <c r="R10">
-        <v>4.37</v>
+        <v>0.529</v>
       </c>
       <c r="S10">
-        <v>5.25</v>
+        <v>0.729</v>
       </c>
       <c r="T10">
-        <v>4.69</v>
+        <v>0.602</v>
       </c>
       <c r="U10">
-        <v>4.18</v>
+        <v>0.628</v>
       </c>
       <c r="V10">
-        <v>4.5</v>
+        <v>0.662</v>
       </c>
       <c r="Y10" s="2" t="s">
         <v>13</v>
       </c>
       <c r="Z10">
-        <v>4.37</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="AA10">
-        <v>5.25</v>
+        <v>0.706</v>
       </c>
       <c r="AB10">
-        <v>4.69</v>
+        <v>0.602</v>
       </c>
       <c r="AC10">
-        <v>4.03</v>
+        <v>0.628</v>
       </c>
       <c r="AD10">
-        <v>4.5</v>
+        <v>0.662</v>
       </c>
     </row>
     <row r="11" spans="1:30">
@@ -1073,73 +1076,73 @@
         <v>14</v>
       </c>
       <c r="B11">
-        <v>2887</v>
+        <v>5.45</v>
       </c>
       <c r="C11">
-        <v>4912</v>
+        <v>6.31</v>
       </c>
       <c r="D11">
-        <v>1856</v>
+        <v>5.52</v>
       </c>
       <c r="E11">
-        <v>10750</v>
+        <v>5.01</v>
       </c>
       <c r="F11">
-        <v>4504</v>
+        <v>5.55</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>14</v>
       </c>
       <c r="J11">
-        <v>2887</v>
+        <v>5.24</v>
       </c>
       <c r="K11">
-        <v>4912</v>
+        <v>6.31</v>
       </c>
       <c r="L11">
-        <v>1856</v>
+        <v>5.52</v>
       </c>
       <c r="M11">
-        <v>10750</v>
+        <v>5.01</v>
       </c>
       <c r="N11">
-        <v>4504</v>
+        <v>5.55</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>14</v>
       </c>
       <c r="R11">
-        <v>2887</v>
+        <v>5.04</v>
       </c>
       <c r="S11">
-        <v>4912</v>
+        <v>6.31</v>
       </c>
       <c r="T11">
-        <v>1856</v>
+        <v>5.52</v>
       </c>
       <c r="U11">
-        <v>8461</v>
+        <v>5.02</v>
       </c>
       <c r="V11">
-        <v>4504</v>
+        <v>5.55</v>
       </c>
       <c r="Y11" s="2" t="s">
         <v>14</v>
       </c>
       <c r="Z11">
-        <v>2887</v>
+        <v>5.24</v>
       </c>
       <c r="AA11">
-        <v>4912</v>
+        <v>6.16</v>
       </c>
       <c r="AB11">
-        <v>1856</v>
+        <v>5.52</v>
       </c>
       <c r="AC11">
-        <v>6225</v>
+        <v>5.02</v>
       </c>
       <c r="AD11">
-        <v>4504</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="12" spans="1:30">
@@ -1147,73 +1150,73 @@
         <v>15</v>
       </c>
       <c r="B12">
-        <v>11.78</v>
+        <v>2039</v>
       </c>
       <c r="C12">
-        <v>5.68</v>
+        <v>3282</v>
       </c>
       <c r="D12">
-        <v>10.13</v>
+        <v>1339</v>
       </c>
       <c r="E12">
-        <v>8.92</v>
+        <v>5541</v>
       </c>
       <c r="F12">
-        <v>7.57</v>
+        <v>1566</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J12">
-        <v>9.15</v>
+        <v>1608</v>
       </c>
       <c r="K12">
-        <v>4.17</v>
+        <v>3282</v>
       </c>
       <c r="L12">
-        <v>7.69</v>
+        <v>1339</v>
       </c>
       <c r="M12">
-        <v>6.58</v>
+        <v>5541</v>
       </c>
       <c r="N12">
-        <v>5.56</v>
+        <v>1566</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="R12">
-        <v>7.51</v>
+        <v>1758</v>
       </c>
       <c r="S12">
-        <v>3.24</v>
+        <v>3282</v>
       </c>
       <c r="T12">
-        <v>6.15</v>
+        <v>1339</v>
       </c>
       <c r="U12">
-        <v>5.04</v>
+        <v>4927</v>
       </c>
       <c r="V12">
-        <v>4.33</v>
+        <v>1566</v>
       </c>
       <c r="Y12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="Z12">
-        <v>6.92</v>
+        <v>1608</v>
       </c>
       <c r="AA12">
-        <v>2.95</v>
+        <v>3229</v>
       </c>
       <c r="AB12">
-        <v>5.61</v>
+        <v>1339</v>
       </c>
       <c r="AC12">
-        <v>4.47</v>
+        <v>4927</v>
       </c>
       <c r="AD12">
-        <v>3.95</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="13" spans="1:30">
@@ -1221,73 +1224,73 @@
         <v>16</v>
       </c>
       <c r="B13">
-        <v>9.710000000000001</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="C13">
-        <v>5.36</v>
+        <v>4.67</v>
       </c>
       <c r="D13">
-        <v>8.800000000000001</v>
+        <v>7.34</v>
       </c>
       <c r="E13">
-        <v>8.52</v>
+        <v>6.41</v>
       </c>
       <c r="F13">
-        <v>7.16</v>
+        <v>5.89</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>16</v>
       </c>
       <c r="J13">
-        <v>7.04</v>
+        <v>7.4</v>
       </c>
       <c r="K13">
-        <v>3.84</v>
+        <v>4.04</v>
       </c>
       <c r="L13">
-        <v>6.34</v>
+        <v>6.5</v>
       </c>
       <c r="M13">
-        <v>6.17</v>
+        <v>5.58</v>
       </c>
       <c r="N13">
-        <v>5.15</v>
+        <v>5.13</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>16</v>
       </c>
       <c r="R13">
-        <v>5.37</v>
+        <v>5.98</v>
       </c>
       <c r="S13">
-        <v>2.94</v>
+        <v>3.13</v>
       </c>
       <c r="T13">
-        <v>4.81</v>
+        <v>5.24</v>
       </c>
       <c r="U13">
-        <v>4.7</v>
+        <v>4.3</v>
       </c>
       <c r="V13">
-        <v>3.94</v>
+        <v>3.98</v>
       </c>
       <c r="Y13" s="2" t="s">
         <v>16</v>
       </c>
       <c r="Z13">
-        <v>4.76</v>
+        <v>5.34</v>
       </c>
       <c r="AA13">
-        <v>2.66</v>
+        <v>2.76</v>
       </c>
       <c r="AB13">
-        <v>4.25</v>
+        <v>4.7</v>
       </c>
       <c r="AC13">
-        <v>4.17</v>
+        <v>3.77</v>
       </c>
       <c r="AD13">
-        <v>3.57</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="14" spans="1:30">
@@ -1295,73 +1298,73 @@
         <v>17</v>
       </c>
       <c r="B14">
-        <v>1549</v>
+        <v>6.69</v>
       </c>
       <c r="C14">
-        <v>1250</v>
+        <v>4.38</v>
       </c>
       <c r="D14">
-        <v>1470</v>
+        <v>6.26</v>
       </c>
       <c r="E14">
-        <v>1411</v>
+        <v>6.1</v>
       </c>
       <c r="F14">
-        <v>1211</v>
+        <v>5.61</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J14">
-        <v>1377</v>
+        <v>6.08</v>
       </c>
       <c r="K14">
-        <v>1152</v>
+        <v>3.75</v>
       </c>
       <c r="L14">
-        <v>1308</v>
+        <v>5.42</v>
       </c>
       <c r="M14">
-        <v>1257</v>
+        <v>5.27</v>
       </c>
       <c r="N14">
-        <v>1078</v>
+        <v>4.85</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>17</v>
       </c>
       <c r="R14">
-        <v>1267</v>
+        <v>4.57</v>
       </c>
       <c r="S14">
-        <v>1090</v>
+        <v>2.87</v>
       </c>
       <c r="T14">
-        <v>1207</v>
+        <v>4.17</v>
       </c>
       <c r="U14">
-        <v>1154</v>
+        <v>4.03</v>
       </c>
       <c r="V14">
-        <v>997</v>
+        <v>3.72</v>
       </c>
       <c r="Y14" s="2" t="s">
         <v>17</v>
       </c>
       <c r="Z14">
-        <v>1226</v>
+        <v>4.02</v>
       </c>
       <c r="AA14">
-        <v>1070</v>
+        <v>2.5</v>
       </c>
       <c r="AB14">
-        <v>1169</v>
+        <v>3.62</v>
       </c>
       <c r="AC14">
-        <v>1114</v>
+        <v>3.5</v>
       </c>
       <c r="AD14">
-        <v>970</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="15" spans="1:30">
@@ -1369,2001 +1372,2223 @@
         <v>18</v>
       </c>
       <c r="B15">
-        <v>2.443</v>
+        <v>1316</v>
       </c>
       <c r="C15">
-        <v>1.222</v>
+        <v>1183</v>
       </c>
       <c r="D15">
-        <v>2.11</v>
+        <v>1283</v>
       </c>
       <c r="E15">
-        <v>1.869</v>
+        <v>1243</v>
       </c>
       <c r="F15">
-        <v>1.599</v>
+        <v>1098</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>18</v>
       </c>
       <c r="J15">
-        <v>1.919</v>
+        <v>1260</v>
       </c>
       <c r="K15">
-        <v>0.921</v>
+        <v>1143</v>
       </c>
       <c r="L15">
-        <v>1.623</v>
+        <v>1229</v>
       </c>
       <c r="M15">
-        <v>1.402</v>
+        <v>1190</v>
       </c>
       <c r="N15">
-        <v>1.198</v>
+        <v>1050</v>
       </c>
       <c r="Q15" s="2" t="s">
         <v>18</v>
       </c>
       <c r="R15">
-        <v>1.592</v>
+        <v>1166</v>
       </c>
       <c r="S15">
-        <v>0.737</v>
+        <v>1083</v>
       </c>
       <c r="T15">
-        <v>1.317</v>
+        <v>1145</v>
       </c>
       <c r="U15">
-        <v>1.097</v>
+        <v>1104</v>
       </c>
       <c r="V15">
-        <v>0.953</v>
+        <v>973</v>
       </c>
       <c r="Y15" s="2" t="s">
         <v>18</v>
       </c>
       <c r="Z15">
-        <v>1.475</v>
+        <v>1121</v>
       </c>
       <c r="AA15">
-        <v>0.68</v>
+        <v>1058</v>
       </c>
       <c r="AB15">
-        <v>1.209</v>
+        <v>1108</v>
       </c>
       <c r="AC15">
-        <v>0.982</v>
+        <v>1067</v>
       </c>
       <c r="AD15">
-        <v>0.878</v>
-      </c>
-    </row>
-    <row r="18" spans="1:30">
-      <c r="A18" s="1" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30">
+      <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="B16">
+        <v>1.746</v>
+      </c>
+      <c r="C16">
+        <v>1.02</v>
+      </c>
+      <c r="D16">
+        <v>1.553</v>
+      </c>
+      <c r="E16">
+        <v>1.367</v>
+      </c>
+      <c r="F16">
+        <v>1.263</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="Q18" s="1" t="s">
+      <c r="J16">
+        <v>1.57</v>
+      </c>
+      <c r="K16">
+        <v>0.896</v>
+      </c>
+      <c r="L16">
+        <v>1.386</v>
+      </c>
+      <c r="M16">
+        <v>1.202</v>
+      </c>
+      <c r="N16">
+        <v>1.112</v>
+      </c>
+      <c r="Q16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="Y18" s="1" t="s">
+      <c r="R16">
+        <v>1.288</v>
+      </c>
+      <c r="S16">
+        <v>0.715</v>
+      </c>
+      <c r="T16">
+        <v>1.135</v>
+      </c>
+      <c r="U16">
+        <v>0.948</v>
+      </c>
+      <c r="V16">
+        <v>0.883</v>
+      </c>
+      <c r="Y16" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="Z16">
+        <v>1.16</v>
+      </c>
+      <c r="AA16">
+        <v>0.642</v>
+      </c>
+      <c r="AB16">
+        <v>1.027</v>
+      </c>
+      <c r="AC16">
+        <v>0.843</v>
+      </c>
+      <c r="AD16">
+        <v>0.785</v>
+      </c>
     </row>
     <row r="19" spans="1:30">
-      <c r="B19" s="2" t="s">
+      <c r="A19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y19" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30">
+      <c r="B20" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="K20" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="L20" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M19" s="2" t="s">
+      <c r="M20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="N19" s="2" t="s">
+      <c r="N20" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="R19" s="2" t="s">
+      <c r="R20" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="S19" s="2" t="s">
+      <c r="S20" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="T19" s="2" t="s">
+      <c r="T20" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="U19" s="2" t="s">
+      <c r="U20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="V19" s="2" t="s">
+      <c r="V20" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="Z19" s="2" t="s">
+      <c r="Z20" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="AA19" s="2" t="s">
+      <c r="AA20" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="AB19" s="2" t="s">
+      <c r="AB20" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="AC19" s="2" t="s">
+      <c r="AC20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="AD19" s="2" t="s">
+      <c r="AD20" s="2" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:30">
-      <c r="A20" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20">
-        <v>870</v>
-      </c>
-      <c r="C20">
-        <v>1002</v>
-      </c>
-      <c r="D20">
-        <v>838</v>
-      </c>
-      <c r="E20">
-        <v>1284</v>
-      </c>
-      <c r="F20">
-        <v>1248</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J20">
-        <v>870</v>
-      </c>
-      <c r="K20">
-        <v>1002</v>
-      </c>
-      <c r="L20">
-        <v>838</v>
-      </c>
-      <c r="M20">
-        <v>1284</v>
-      </c>
-      <c r="N20">
-        <v>1248</v>
-      </c>
-      <c r="Q20" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="R20">
-        <v>870</v>
-      </c>
-      <c r="S20">
-        <v>1002</v>
-      </c>
-      <c r="T20">
-        <v>838</v>
-      </c>
-      <c r="U20">
-        <v>1146</v>
-      </c>
-      <c r="V20">
-        <v>1248</v>
-      </c>
-      <c r="Y20" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="Z20">
-        <v>870</v>
-      </c>
-      <c r="AA20">
-        <v>1002</v>
-      </c>
-      <c r="AB20">
-        <v>838</v>
-      </c>
-      <c r="AC20">
-        <v>882</v>
-      </c>
-      <c r="AD20">
-        <v>1248</v>
       </c>
     </row>
     <row r="21" spans="1:30">
       <c r="A21" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B21">
-        <v>800</v>
+        <v>20</v>
       </c>
       <c r="C21">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="D21">
-        <v>700</v>
+        <v>10</v>
       </c>
       <c r="E21">
-        <v>300</v>
+        <v>10</v>
       </c>
       <c r="F21">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J21">
-        <v>800</v>
+        <v>20</v>
       </c>
       <c r="K21">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="L21">
-        <v>700</v>
+        <v>10</v>
       </c>
       <c r="M21">
-        <v>300</v>
+        <v>10</v>
       </c>
       <c r="N21">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R21">
-        <v>800</v>
+        <v>10</v>
       </c>
       <c r="S21">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="T21">
-        <v>700</v>
+        <v>10</v>
       </c>
       <c r="U21">
-        <v>500</v>
+        <v>10</v>
       </c>
       <c r="V21">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="Y21" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Z21">
-        <v>800</v>
+        <v>20</v>
       </c>
       <c r="AA21">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="AB21">
-        <v>700</v>
+        <v>10</v>
       </c>
       <c r="AC21">
-        <v>900</v>
+        <v>10</v>
       </c>
       <c r="AD21">
-        <v>100</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:30">
       <c r="A22" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>822</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>888</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>722</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>1032</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>930</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J22">
-        <v>0</v>
+        <v>696</v>
       </c>
       <c r="K22">
-        <v>0</v>
+        <v>888</v>
       </c>
       <c r="L22">
-        <v>0</v>
+        <v>722</v>
       </c>
       <c r="M22">
-        <v>0</v>
+        <v>1032</v>
       </c>
       <c r="N22">
-        <v>0</v>
+        <v>930</v>
       </c>
       <c r="Q22" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R22">
-        <v>0</v>
+        <v>690</v>
       </c>
       <c r="S22">
-        <v>0</v>
+        <v>888</v>
       </c>
       <c r="T22">
-        <v>0</v>
+        <v>722</v>
       </c>
       <c r="U22">
-        <v>0</v>
+        <v>888</v>
       </c>
       <c r="V22">
-        <v>0</v>
+        <v>930</v>
       </c>
       <c r="Y22" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Z22">
-        <v>0</v>
+        <v>696</v>
       </c>
       <c r="AA22">
-        <v>0</v>
+        <v>756</v>
       </c>
       <c r="AB22">
-        <v>0</v>
+        <v>722</v>
       </c>
       <c r="AC22">
-        <v>0</v>
+        <v>888</v>
       </c>
       <c r="AD22">
-        <v>0</v>
+        <v>930</v>
       </c>
     </row>
     <row r="23" spans="1:30">
       <c r="A23" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="K23">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="L23">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="M23">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="N23">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="Q23" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="R23">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="S23">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="T23">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="U23">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="V23">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="Y23" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Z23">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="AA23">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="AB23">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="AC23">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="AD23">
-        <v>0</v>
+        <v>800</v>
       </c>
     </row>
     <row r="24" spans="1:30">
       <c r="A24" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B24">
-        <v>1320</v>
+        <v>114</v>
       </c>
       <c r="C24">
-        <v>800</v>
+        <v>96</v>
       </c>
       <c r="D24">
-        <v>1240</v>
+        <v>120</v>
       </c>
       <c r="E24">
-        <v>1160</v>
+        <v>108</v>
       </c>
       <c r="F24">
-        <v>1000</v>
+        <v>108</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J24">
-        <v>1320</v>
+        <v>126</v>
       </c>
       <c r="K24">
-        <v>800</v>
+        <v>96</v>
       </c>
       <c r="L24">
-        <v>1240</v>
+        <v>120</v>
       </c>
       <c r="M24">
-        <v>1160</v>
+        <v>108</v>
       </c>
       <c r="N24">
-        <v>1000</v>
+        <v>108</v>
       </c>
       <c r="Q24" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="R24">
-        <v>1320</v>
+        <v>138</v>
       </c>
       <c r="S24">
-        <v>800</v>
+        <v>96</v>
       </c>
       <c r="T24">
-        <v>1240</v>
+        <v>120</v>
       </c>
       <c r="U24">
-        <v>1240</v>
+        <v>114</v>
       </c>
       <c r="V24">
-        <v>1000</v>
+        <v>108</v>
       </c>
       <c r="Y24" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Z24">
-        <v>1320</v>
+        <v>126</v>
       </c>
       <c r="AA24">
-        <v>800</v>
+        <v>102</v>
       </c>
       <c r="AB24">
-        <v>1240</v>
+        <v>120</v>
       </c>
       <c r="AC24">
-        <v>1400</v>
+        <v>114</v>
       </c>
       <c r="AD24">
-        <v>1000</v>
+        <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:30">
       <c r="A25" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B25">
-        <v>0.387</v>
+        <v>1</v>
       </c>
       <c r="C25">
-        <v>0.612</v>
+        <v>1</v>
       </c>
       <c r="D25">
-        <v>0.415</v>
+        <v>1</v>
       </c>
       <c r="E25">
-        <v>0.433</v>
+        <v>1</v>
       </c>
       <c r="F25">
-        <v>0.492</v>
+        <v>1</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J25">
-        <v>0.387</v>
+        <v>1</v>
       </c>
       <c r="K25">
-        <v>0.612</v>
+        <v>1</v>
       </c>
       <c r="L25">
-        <v>0.415</v>
+        <v>1</v>
       </c>
       <c r="M25">
-        <v>0.433</v>
+        <v>1</v>
       </c>
       <c r="N25">
-        <v>0.492</v>
+        <v>1</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="R25">
-        <v>0.387</v>
+        <v>1</v>
       </c>
       <c r="S25">
-        <v>0.612</v>
+        <v>1</v>
       </c>
       <c r="T25">
-        <v>0.415</v>
+        <v>1</v>
       </c>
       <c r="U25">
-        <v>0.409</v>
+        <v>1</v>
       </c>
       <c r="V25">
-        <v>0.492</v>
+        <v>1</v>
       </c>
       <c r="Y25" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Z25">
-        <v>0.387</v>
+        <v>1</v>
       </c>
       <c r="AA25">
-        <v>0.612</v>
+        <v>1</v>
       </c>
       <c r="AB25">
-        <v>0.415</v>
+        <v>1</v>
       </c>
       <c r="AC25">
-        <v>0.365</v>
+        <v>1</v>
       </c>
       <c r="AD25">
-        <v>0.492</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:30">
       <c r="A26" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26">
-        <v>4.37</v>
+        <v>760</v>
       </c>
       <c r="C26">
-        <v>5.25</v>
+        <v>640</v>
       </c>
       <c r="D26">
-        <v>4.69</v>
+        <v>800</v>
       </c>
       <c r="E26">
-        <v>4.09</v>
+        <v>720</v>
       </c>
       <c r="F26">
-        <v>4.5</v>
+        <v>720</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J26">
-        <v>4.37</v>
+        <v>840</v>
       </c>
       <c r="K26">
-        <v>5.25</v>
+        <v>640</v>
       </c>
       <c r="L26">
-        <v>4.69</v>
+        <v>800</v>
       </c>
       <c r="M26">
-        <v>4.09</v>
+        <v>720</v>
       </c>
       <c r="N26">
-        <v>4.5</v>
+        <v>720</v>
       </c>
       <c r="Q26" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="R26">
-        <v>4.37</v>
+        <v>920</v>
       </c>
       <c r="S26">
-        <v>5.25</v>
+        <v>640</v>
       </c>
       <c r="T26">
-        <v>4.69</v>
+        <v>800</v>
       </c>
       <c r="U26">
-        <v>4.18</v>
+        <v>760</v>
       </c>
       <c r="V26">
-        <v>4.5</v>
+        <v>720</v>
       </c>
       <c r="Y26" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Z26">
-        <v>4.37</v>
+        <v>840</v>
       </c>
       <c r="AA26">
-        <v>5.25</v>
+        <v>680</v>
       </c>
       <c r="AB26">
-        <v>4.69</v>
+        <v>800</v>
       </c>
       <c r="AC26">
-        <v>4.03</v>
+        <v>760</v>
       </c>
       <c r="AD26">
-        <v>4.5</v>
+        <v>720</v>
       </c>
     </row>
     <row r="27" spans="1:30">
       <c r="A27" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B27">
-        <v>2887</v>
+        <v>0.628</v>
       </c>
       <c r="C27">
-        <v>4912</v>
+        <v>0.729</v>
       </c>
       <c r="D27">
-        <v>1856</v>
+        <v>0.602</v>
       </c>
       <c r="E27">
-        <v>10750</v>
+        <v>0.65</v>
       </c>
       <c r="F27">
-        <v>4504</v>
+        <v>0.662</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J27">
-        <v>2887</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="K27">
-        <v>4912</v>
+        <v>0.729</v>
       </c>
       <c r="L27">
-        <v>1856</v>
+        <v>0.602</v>
       </c>
       <c r="M27">
-        <v>10750</v>
+        <v>0.65</v>
       </c>
       <c r="N27">
-        <v>4504</v>
+        <v>0.662</v>
       </c>
       <c r="Q27" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R27">
-        <v>2887</v>
+        <v>0.529</v>
       </c>
       <c r="S27">
-        <v>4912</v>
+        <v>0.729</v>
       </c>
       <c r="T27">
-        <v>1856</v>
+        <v>0.602</v>
       </c>
       <c r="U27">
-        <v>9225</v>
+        <v>0.628</v>
       </c>
       <c r="V27">
-        <v>4504</v>
+        <v>0.662</v>
       </c>
       <c r="Y27" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Z27">
-        <v>2887</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="AA27">
-        <v>4912</v>
+        <v>0.706</v>
       </c>
       <c r="AB27">
-        <v>1856</v>
+        <v>0.602</v>
       </c>
       <c r="AC27">
-        <v>6225</v>
+        <v>0.628</v>
       </c>
       <c r="AD27">
-        <v>4504</v>
+        <v>0.662</v>
       </c>
     </row>
     <row r="28" spans="1:30">
       <c r="A28" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B28">
-        <v>10.79</v>
+        <v>5.45</v>
       </c>
       <c r="C28">
-        <v>4.86</v>
+        <v>6.31</v>
       </c>
       <c r="D28">
-        <v>9.210000000000001</v>
+        <v>5.52</v>
       </c>
       <c r="E28">
-        <v>8.109999999999999</v>
+        <v>5.01</v>
       </c>
       <c r="F28">
-        <v>6.74</v>
+        <v>5.55</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J28">
-        <v>8.17</v>
+        <v>5.24</v>
       </c>
       <c r="K28">
-        <v>3.36</v>
+        <v>6.31</v>
       </c>
       <c r="L28">
-        <v>6.78</v>
+        <v>5.52</v>
       </c>
       <c r="M28">
-        <v>5.79</v>
+        <v>5.01</v>
       </c>
       <c r="N28">
-        <v>4.74</v>
+        <v>5.55</v>
       </c>
       <c r="Q28" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R28">
-        <v>6.55</v>
+        <v>5.04</v>
       </c>
       <c r="S28">
-        <v>2.45</v>
+        <v>6.31</v>
       </c>
       <c r="T28">
-        <v>5.28</v>
+        <v>5.52</v>
       </c>
       <c r="U28">
-        <v>4.28</v>
+        <v>5.02</v>
       </c>
       <c r="V28">
-        <v>3.54</v>
+        <v>5.55</v>
       </c>
       <c r="Y28" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Z28">
-        <v>6.92</v>
+        <v>5.24</v>
       </c>
       <c r="AA28">
-        <v>2.95</v>
+        <v>6.16</v>
       </c>
       <c r="AB28">
-        <v>5.61</v>
+        <v>5.52</v>
       </c>
       <c r="AC28">
-        <v>4.47</v>
+        <v>5.02</v>
       </c>
       <c r="AD28">
-        <v>3.95</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="29" spans="1:30">
       <c r="A29" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B29">
-        <v>8.789999999999999</v>
+        <v>2039</v>
       </c>
       <c r="C29">
-        <v>4.55</v>
+        <v>3282</v>
       </c>
       <c r="D29">
-        <v>7.93</v>
+        <v>1339</v>
       </c>
       <c r="E29">
-        <v>7.72</v>
+        <v>5541</v>
       </c>
       <c r="F29">
-        <v>6.35</v>
+        <v>1566</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J29">
-        <v>6.17</v>
+        <v>1608</v>
       </c>
       <c r="K29">
-        <v>3.05</v>
+        <v>3282</v>
       </c>
       <c r="L29">
-        <v>5.51</v>
+        <v>1339</v>
       </c>
       <c r="M29">
-        <v>5.39</v>
+        <v>5541</v>
       </c>
       <c r="N29">
-        <v>4.35</v>
+        <v>1566</v>
       </c>
       <c r="Q29" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="R29">
-        <v>4.54</v>
+        <v>1758</v>
       </c>
       <c r="S29">
-        <v>2.17</v>
+        <v>3282</v>
       </c>
       <c r="T29">
-        <v>4.01</v>
+        <v>1339</v>
       </c>
       <c r="U29">
-        <v>3.94</v>
+        <v>4927</v>
       </c>
       <c r="V29">
-        <v>3.17</v>
+        <v>1566</v>
       </c>
       <c r="Y29" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Z29">
-        <v>4.76</v>
+        <v>1608</v>
       </c>
       <c r="AA29">
-        <v>2.66</v>
+        <v>3229</v>
       </c>
       <c r="AB29">
-        <v>4.25</v>
+        <v>1339</v>
       </c>
       <c r="AC29">
-        <v>4.17</v>
+        <v>4927</v>
       </c>
       <c r="AD29">
-        <v>3.57</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="30" spans="1:30">
       <c r="A30" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B30">
-        <v>1483</v>
+        <v>7.32</v>
       </c>
       <c r="C30">
-        <v>1196</v>
+        <v>3.86</v>
       </c>
       <c r="D30">
-        <v>1408</v>
+        <v>6.45</v>
       </c>
       <c r="E30">
-        <v>1357</v>
+        <v>5.62</v>
       </c>
       <c r="F30">
-        <v>1155</v>
+        <v>5.07</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J30">
-        <v>1312</v>
+        <v>6.48</v>
       </c>
       <c r="K30">
-        <v>1098</v>
+        <v>3.24</v>
       </c>
       <c r="L30">
-        <v>1248</v>
+        <v>5.62</v>
       </c>
       <c r="M30">
-        <v>1204</v>
+        <v>4.8</v>
       </c>
       <c r="N30">
-        <v>1024</v>
+        <v>4.33</v>
       </c>
       <c r="Q30" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="R30">
-        <v>1204</v>
+        <v>5.1</v>
       </c>
       <c r="S30">
-        <v>1038</v>
+        <v>2.36</v>
       </c>
       <c r="T30">
-        <v>1148</v>
+        <v>4.39</v>
       </c>
       <c r="U30">
-        <v>1103</v>
+        <v>3.57</v>
       </c>
       <c r="V30">
-        <v>944</v>
+        <v>3.21</v>
       </c>
       <c r="Y30" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Z30">
-        <v>1226</v>
+        <v>5.34</v>
       </c>
       <c r="AA30">
-        <v>1070</v>
+        <v>2.76</v>
       </c>
       <c r="AB30">
-        <v>1169</v>
+        <v>4.7</v>
       </c>
       <c r="AC30">
-        <v>1114</v>
+        <v>3.77</v>
       </c>
       <c r="AD30">
-        <v>970</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="31" spans="1:30">
       <c r="A31" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B31">
+        <v>5.81</v>
+      </c>
+      <c r="C31">
+        <v>3.58</v>
+      </c>
+      <c r="D31">
+        <v>5.42</v>
+      </c>
+      <c r="E31">
+        <v>5.32</v>
+      </c>
+      <c r="F31">
+        <v>4.8</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J31">
+        <v>5.23</v>
+      </c>
+      <c r="K31">
+        <v>2.96</v>
+      </c>
+      <c r="L31">
+        <v>4.6</v>
+      </c>
+      <c r="M31">
+        <v>4.5</v>
+      </c>
+      <c r="N31">
+        <v>4.05</v>
+      </c>
+      <c r="Q31" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R31">
+        <v>3.78</v>
+      </c>
+      <c r="S31">
+        <v>2.1</v>
+      </c>
+      <c r="T31">
+        <v>3.39</v>
+      </c>
+      <c r="U31">
+        <v>3.3</v>
+      </c>
+      <c r="V31">
+        <v>2.97</v>
+      </c>
+      <c r="Y31" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z31">
+        <v>4.02</v>
+      </c>
+      <c r="AA31">
+        <v>2.5</v>
+      </c>
+      <c r="AB31">
+        <v>3.62</v>
+      </c>
+      <c r="AC31">
+        <v>3.5</v>
+      </c>
+      <c r="AD31">
+        <v>3.23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:30">
+      <c r="A32" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B31">
-        <v>2.245</v>
-      </c>
-      <c r="C31">
-        <v>1.059</v>
-      </c>
-      <c r="D31">
-        <v>1.926</v>
-      </c>
-      <c r="E31">
-        <v>1.708</v>
-      </c>
-      <c r="F31">
-        <v>1.434</v>
-      </c>
-      <c r="I31" s="2" t="s">
+      <c r="B32">
+        <v>1252</v>
+      </c>
+      <c r="C32">
+        <v>1129</v>
+      </c>
+      <c r="D32">
+        <v>1224</v>
+      </c>
+      <c r="E32">
+        <v>1190</v>
+      </c>
+      <c r="F32">
+        <v>1044</v>
+      </c>
+      <c r="I32" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J31">
-        <v>1.724</v>
-      </c>
-      <c r="K31">
-        <v>0.761</v>
-      </c>
-      <c r="L31">
-        <v>1.443</v>
-      </c>
-      <c r="M31">
-        <v>1.245</v>
-      </c>
-      <c r="N31">
-        <v>1.036</v>
-      </c>
-      <c r="Q31" s="2" t="s">
+      <c r="J32">
+        <v>1199</v>
+      </c>
+      <c r="K32">
+        <v>1090</v>
+      </c>
+      <c r="L32">
+        <v>1171</v>
+      </c>
+      <c r="M32">
+        <v>1138</v>
+      </c>
+      <c r="N32">
+        <v>996</v>
+      </c>
+      <c r="Q32" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="R31">
-        <v>1.401</v>
-      </c>
-      <c r="S31">
-        <v>0.58</v>
-      </c>
-      <c r="T31">
-        <v>1.142</v>
-      </c>
-      <c r="U31">
-        <v>0.945</v>
-      </c>
-      <c r="V31">
-        <v>0.795</v>
-      </c>
-      <c r="Y31" s="2" t="s">
+      <c r="R32">
+        <v>1107</v>
+      </c>
+      <c r="S32">
+        <v>1032</v>
+      </c>
+      <c r="T32">
+        <v>1089</v>
+      </c>
+      <c r="U32">
+        <v>1056</v>
+      </c>
+      <c r="V32">
+        <v>922</v>
+      </c>
+      <c r="Y32" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Z31">
-        <v>1.475</v>
-      </c>
-      <c r="AA31">
-        <v>0.68</v>
-      </c>
-      <c r="AB31">
-        <v>1.209</v>
-      </c>
-      <c r="AC31">
-        <v>0.982</v>
-      </c>
-      <c r="AD31">
-        <v>0.878</v>
-      </c>
-    </row>
-    <row r="34" spans="1:30">
-      <c r="A34" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q34" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y34" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="35" spans="1:30">
-      <c r="B35" s="2" t="s">
+      <c r="Z32">
+        <v>1121</v>
+      </c>
+      <c r="AA32">
+        <v>1058</v>
+      </c>
+      <c r="AB32">
+        <v>1108</v>
+      </c>
+      <c r="AC32">
+        <v>1067</v>
+      </c>
+      <c r="AD32">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="33" spans="1:30">
+      <c r="A33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33">
+        <v>1.554</v>
+      </c>
+      <c r="C33">
+        <v>0.859</v>
+      </c>
+      <c r="D33">
+        <v>1.375</v>
+      </c>
+      <c r="E33">
+        <v>1.21</v>
+      </c>
+      <c r="F33">
+        <v>1.1</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J33">
+        <v>1.386</v>
+      </c>
+      <c r="K33">
+        <v>0.736</v>
+      </c>
+      <c r="L33">
+        <v>1.211</v>
+      </c>
+      <c r="M33">
+        <v>1.048</v>
+      </c>
+      <c r="N33">
+        <v>0.952</v>
+      </c>
+      <c r="Q33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="R33">
+        <v>1.112</v>
+      </c>
+      <c r="S33">
+        <v>0.5610000000000001</v>
+      </c>
+      <c r="T33">
+        <v>0.965</v>
+      </c>
+      <c r="U33">
+        <v>0.802</v>
+      </c>
+      <c r="V33">
+        <v>0.731</v>
+      </c>
+      <c r="Y33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="Z33">
+        <v>1.16</v>
+      </c>
+      <c r="AA33">
+        <v>0.642</v>
+      </c>
+      <c r="AB33">
+        <v>1.027</v>
+      </c>
+      <c r="AC33">
+        <v>0.843</v>
+      </c>
+      <c r="AD33">
+        <v>0.785</v>
+      </c>
+    </row>
+    <row r="36" spans="1:30">
+      <c r="A36" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q36" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y36" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:30">
+      <c r="B37" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D37" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E37" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J35" s="2" t="s">
+      <c r="J37" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="K35" s="2" t="s">
+      <c r="K37" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="L35" s="2" t="s">
+      <c r="L37" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M35" s="2" t="s">
+      <c r="M37" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="N35" s="2" t="s">
+      <c r="N37" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="R35" s="2" t="s">
+      <c r="R37" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="S35" s="2" t="s">
+      <c r="S37" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="T35" s="2" t="s">
+      <c r="T37" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="U35" s="2" t="s">
+      <c r="U37" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="V35" s="2" t="s">
+      <c r="V37" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="Z35" s="2" t="s">
+      <c r="Z37" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="AA35" s="2" t="s">
+      <c r="AA37" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="AB35" s="2" t="s">
+      <c r="AB37" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="AC35" s="2" t="s">
+      <c r="AC37" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="AD35" s="2" t="s">
+      <c r="AD37" s="2" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="36" spans="1:30">
-      <c r="A36" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B36">
-        <v>930</v>
-      </c>
-      <c r="C36">
-        <v>1002</v>
-      </c>
-      <c r="D36">
-        <v>888</v>
-      </c>
-      <c r="E36">
-        <v>1284</v>
-      </c>
-      <c r="F36">
-        <v>1248</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J36">
-        <v>870</v>
-      </c>
-      <c r="K36">
-        <v>1002</v>
-      </c>
-      <c r="L36">
-        <v>838</v>
-      </c>
-      <c r="M36">
-        <v>1284</v>
-      </c>
-      <c r="N36">
-        <v>1248</v>
-      </c>
-      <c r="Q36" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="R36">
-        <v>870</v>
-      </c>
-      <c r="S36">
-        <v>1002</v>
-      </c>
-      <c r="T36">
-        <v>838</v>
-      </c>
-      <c r="U36">
-        <v>1284</v>
-      </c>
-      <c r="V36">
-        <v>1248</v>
-      </c>
-      <c r="Y36" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="Z36">
-        <v>870</v>
-      </c>
-      <c r="AA36">
-        <v>1002</v>
-      </c>
-      <c r="AB36">
-        <v>838</v>
-      </c>
-      <c r="AC36">
-        <v>882</v>
-      </c>
-      <c r="AD36">
-        <v>1248</v>
-      </c>
-    </row>
-    <row r="37" spans="1:30">
-      <c r="A37" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B37">
-        <v>700</v>
-      </c>
-      <c r="C37">
-        <v>100</v>
-      </c>
-      <c r="D37">
-        <v>600</v>
-      </c>
-      <c r="E37">
-        <v>300</v>
-      </c>
-      <c r="F37">
-        <v>100</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J37">
-        <v>800</v>
-      </c>
-      <c r="K37">
-        <v>100</v>
-      </c>
-      <c r="L37">
-        <v>700</v>
-      </c>
-      <c r="M37">
-        <v>300</v>
-      </c>
-      <c r="N37">
-        <v>100</v>
-      </c>
-      <c r="Q37" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="R37">
-        <v>800</v>
-      </c>
-      <c r="S37">
-        <v>100</v>
-      </c>
-      <c r="T37">
-        <v>700</v>
-      </c>
-      <c r="U37">
-        <v>300</v>
-      </c>
-      <c r="V37">
-        <v>100</v>
-      </c>
-      <c r="Y37" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="Z37">
-        <v>800</v>
-      </c>
-      <c r="AA37">
-        <v>100</v>
-      </c>
-      <c r="AB37">
-        <v>700</v>
-      </c>
-      <c r="AC37">
-        <v>900</v>
-      </c>
-      <c r="AD37">
-        <v>100</v>
       </c>
     </row>
     <row r="38" spans="1:30">
       <c r="A38" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B38">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C38">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="D38">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J38">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K38">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L38">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q38" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="R38">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="S38">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="T38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y38" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Z38">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="AA38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AB38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AC38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AD38">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:30">
       <c r="A39" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B39">
-        <v>0</v>
+        <v>1080</v>
       </c>
       <c r="C39">
-        <v>0</v>
+        <v>1098</v>
       </c>
       <c r="D39">
-        <v>0</v>
+        <v>838</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>1032</v>
       </c>
       <c r="F39">
-        <v>0</v>
+        <v>1056</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J39">
-        <v>0</v>
+        <v>822</v>
       </c>
       <c r="K39">
-        <v>0</v>
+        <v>1230</v>
       </c>
       <c r="L39">
-        <v>0</v>
+        <v>838</v>
       </c>
       <c r="M39">
-        <v>0</v>
+        <v>1032</v>
       </c>
       <c r="N39">
-        <v>0</v>
+        <v>1056</v>
       </c>
       <c r="Q39" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="R39">
-        <v>0</v>
+        <v>822</v>
       </c>
       <c r="S39">
-        <v>0</v>
+        <v>1230</v>
       </c>
       <c r="T39">
-        <v>0</v>
+        <v>722</v>
       </c>
       <c r="U39">
-        <v>0</v>
+        <v>1032</v>
       </c>
       <c r="V39">
-        <v>0</v>
+        <v>1176</v>
       </c>
       <c r="Y39" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Z39">
-        <v>0</v>
+        <v>696</v>
       </c>
       <c r="AA39">
-        <v>0</v>
+        <v>756</v>
       </c>
       <c r="AB39">
-        <v>0</v>
+        <v>722</v>
       </c>
       <c r="AC39">
-        <v>0</v>
+        <v>888</v>
       </c>
       <c r="AD39">
-        <v>0</v>
+        <v>930</v>
       </c>
     </row>
     <row r="40" spans="1:30">
       <c r="A40" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B40">
-        <v>1280</v>
+        <v>1000</v>
       </c>
       <c r="C40">
+        <v>400</v>
+      </c>
+      <c r="D40">
+        <v>1000</v>
+      </c>
+      <c r="E40">
         <v>800</v>
       </c>
-      <c r="D40">
-        <v>1160</v>
-      </c>
-      <c r="E40">
-        <v>1160</v>
-      </c>
       <c r="F40">
+        <v>600</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J40">
+        <v>1200</v>
+      </c>
+      <c r="K40">
+        <v>200</v>
+      </c>
+      <c r="L40">
         <v>1000</v>
       </c>
-      <c r="I40" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J40">
-        <v>1320</v>
-      </c>
-      <c r="K40">
+      <c r="M40">
         <v>800</v>
       </c>
-      <c r="L40">
-        <v>1240</v>
-      </c>
-      <c r="M40">
-        <v>1160</v>
-      </c>
       <c r="N40">
+        <v>600</v>
+      </c>
+      <c r="Q40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="R40">
+        <v>1200</v>
+      </c>
+      <c r="S40">
+        <v>200</v>
+      </c>
+      <c r="T40">
         <v>1000</v>
       </c>
-      <c r="Q40" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="R40">
-        <v>1320</v>
-      </c>
-      <c r="S40">
+      <c r="U40">
         <v>800</v>
       </c>
-      <c r="T40">
-        <v>1240</v>
-      </c>
-      <c r="U40">
-        <v>1160</v>
-      </c>
       <c r="V40">
+        <v>400</v>
+      </c>
+      <c r="Y40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="Z40">
+        <v>1400</v>
+      </c>
+      <c r="AA40">
+        <v>600</v>
+      </c>
+      <c r="AB40">
         <v>1000</v>
       </c>
-      <c r="Y40" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="Z40">
-        <v>1320</v>
-      </c>
-      <c r="AA40">
+      <c r="AC40">
+        <v>1000</v>
+      </c>
+      <c r="AD40">
         <v>800</v>
-      </c>
-      <c r="AB40">
-        <v>1240</v>
-      </c>
-      <c r="AC40">
-        <v>1400</v>
-      </c>
-      <c r="AD40">
-        <v>1000</v>
       </c>
     </row>
     <row r="41" spans="1:30">
       <c r="A41" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B41">
-        <v>0.402</v>
+        <v>96</v>
       </c>
       <c r="C41">
-        <v>0.612</v>
+        <v>90</v>
       </c>
       <c r="D41">
-        <v>0.436</v>
+        <v>102</v>
       </c>
       <c r="E41">
-        <v>0.433</v>
+        <v>108</v>
       </c>
       <c r="F41">
-        <v>0.492</v>
+        <v>102</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J41">
-        <v>0.387</v>
+        <v>114</v>
       </c>
       <c r="K41">
-        <v>0.612</v>
+        <v>96</v>
       </c>
       <c r="L41">
-        <v>0.415</v>
+        <v>102</v>
       </c>
       <c r="M41">
-        <v>0.433</v>
+        <v>108</v>
       </c>
       <c r="N41">
-        <v>0.492</v>
+        <v>102</v>
       </c>
       <c r="Q41" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="R41">
-        <v>0.387</v>
+        <v>114</v>
       </c>
       <c r="S41">
-        <v>0.612</v>
+        <v>96</v>
       </c>
       <c r="T41">
-        <v>0.415</v>
+        <v>120</v>
       </c>
       <c r="U41">
-        <v>0.433</v>
+        <v>108</v>
       </c>
       <c r="V41">
-        <v>0.492</v>
+        <v>108</v>
       </c>
       <c r="Y41" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="Z41">
-        <v>0.387</v>
+        <v>126</v>
       </c>
       <c r="AA41">
-        <v>0.612</v>
+        <v>102</v>
       </c>
       <c r="AB41">
-        <v>0.415</v>
+        <v>120</v>
       </c>
       <c r="AC41">
-        <v>0.365</v>
+        <v>114</v>
       </c>
       <c r="AD41">
-        <v>0.492</v>
+        <v>108</v>
       </c>
     </row>
     <row r="42" spans="1:30">
       <c r="A42" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B42">
-        <v>4.43</v>
+        <v>1</v>
       </c>
       <c r="C42">
-        <v>5.25</v>
+        <v>1</v>
       </c>
       <c r="D42">
-        <v>4.75</v>
+        <v>1</v>
       </c>
       <c r="E42">
-        <v>4.09</v>
+        <v>1</v>
       </c>
       <c r="F42">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J42">
-        <v>4.37</v>
+        <v>1</v>
       </c>
       <c r="K42">
-        <v>5.25</v>
+        <v>1</v>
       </c>
       <c r="L42">
-        <v>4.69</v>
+        <v>1</v>
       </c>
       <c r="M42">
-        <v>4.09</v>
+        <v>1</v>
       </c>
       <c r="N42">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="Q42" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="R42">
-        <v>4.37</v>
+        <v>1</v>
       </c>
       <c r="S42">
-        <v>5.25</v>
+        <v>1</v>
       </c>
       <c r="T42">
-        <v>4.69</v>
+        <v>1</v>
       </c>
       <c r="U42">
-        <v>4.09</v>
+        <v>1</v>
       </c>
       <c r="V42">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="Y42" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="Z42">
-        <v>4.37</v>
+        <v>1</v>
       </c>
       <c r="AA42">
-        <v>5.25</v>
+        <v>1</v>
       </c>
       <c r="AB42">
-        <v>4.69</v>
+        <v>1</v>
       </c>
       <c r="AC42">
-        <v>4.03</v>
+        <v>1</v>
       </c>
       <c r="AD42">
-        <v>4.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:30">
       <c r="A43" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B43">
-        <v>3245</v>
+        <v>640</v>
       </c>
       <c r="C43">
-        <v>4912</v>
+        <v>600</v>
       </c>
       <c r="D43">
-        <v>2479</v>
+        <v>680</v>
       </c>
       <c r="E43">
-        <v>10750</v>
+        <v>720</v>
       </c>
       <c r="F43">
-        <v>4504</v>
+        <v>680</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J43">
-        <v>2887</v>
+        <v>760</v>
       </c>
       <c r="K43">
-        <v>4912</v>
+        <v>640</v>
       </c>
       <c r="L43">
-        <v>1856</v>
+        <v>680</v>
       </c>
       <c r="M43">
-        <v>10750</v>
+        <v>720</v>
       </c>
       <c r="N43">
-        <v>4504</v>
+        <v>680</v>
       </c>
       <c r="Q43" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="R43">
-        <v>2887</v>
+        <v>760</v>
       </c>
       <c r="S43">
-        <v>4912</v>
+        <v>640</v>
       </c>
       <c r="T43">
-        <v>1856</v>
+        <v>800</v>
       </c>
       <c r="U43">
-        <v>10750</v>
+        <v>720</v>
       </c>
       <c r="V43">
-        <v>4504</v>
+        <v>720</v>
       </c>
       <c r="Y43" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="Z43">
-        <v>2887</v>
+        <v>840</v>
       </c>
       <c r="AA43">
-        <v>4912</v>
+        <v>680</v>
       </c>
       <c r="AB43">
-        <v>1856</v>
+        <v>800</v>
       </c>
       <c r="AC43">
-        <v>6225</v>
+        <v>760</v>
       </c>
       <c r="AD43">
-        <v>4504</v>
+        <v>720</v>
       </c>
     </row>
     <row r="44" spans="1:30">
       <c r="A44" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B44">
-        <v>5.58</v>
+        <v>0.72</v>
       </c>
       <c r="C44">
-        <v>1.23</v>
+        <v>0.769</v>
       </c>
       <c r="D44">
-        <v>4.59</v>
+        <v>0.702</v>
       </c>
       <c r="E44">
-        <v>4.45</v>
+        <v>0.65</v>
       </c>
       <c r="F44">
-        <v>3.02</v>
+        <v>0.679</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J44">
-        <v>3.09</v>
+        <v>0.628</v>
       </c>
       <c r="K44">
-        <v>-0.19</v>
+        <v>0.725</v>
       </c>
       <c r="L44">
-        <v>2.28</v>
+        <v>0.702</v>
       </c>
       <c r="M44">
-        <v>2.22</v>
+        <v>0.65</v>
       </c>
       <c r="N44">
-        <v>1.1</v>
+        <v>0.679</v>
       </c>
       <c r="Q44" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="R44">
-        <v>1.64</v>
+        <v>0.628</v>
       </c>
       <c r="S44">
-        <v>-1.02</v>
+        <v>0.725</v>
       </c>
       <c r="T44">
-        <v>0.9399999999999999</v>
+        <v>0.602</v>
       </c>
       <c r="U44">
-        <v>0.8100000000000001</v>
+        <v>0.65</v>
       </c>
       <c r="V44">
-        <v>-0.03</v>
+        <v>0.641</v>
       </c>
       <c r="Y44" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Z44">
-        <v>6.92</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="AA44">
-        <v>2.95</v>
+        <v>0.706</v>
       </c>
       <c r="AB44">
-        <v>5.61</v>
+        <v>0.602</v>
       </c>
       <c r="AC44">
-        <v>4.47</v>
+        <v>0.628</v>
       </c>
       <c r="AD44">
-        <v>3.95</v>
+        <v>0.662</v>
       </c>
     </row>
     <row r="45" spans="1:30">
       <c r="A45" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B45">
-        <v>3.85</v>
+        <v>5.79</v>
       </c>
       <c r="C45">
-        <v>0.95</v>
+        <v>6.7</v>
       </c>
       <c r="D45">
-        <v>3.28</v>
+        <v>5.81</v>
       </c>
       <c r="E45">
-        <v>4.1</v>
+        <v>5.01</v>
       </c>
       <c r="F45">
-        <v>2.68</v>
+        <v>5.59</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J45">
-        <v>1.64</v>
+        <v>5.45</v>
       </c>
       <c r="K45">
-        <v>-0.46</v>
+        <v>6.59</v>
       </c>
       <c r="L45">
-        <v>1.35</v>
+        <v>5.81</v>
       </c>
       <c r="M45">
-        <v>1.88</v>
+        <v>5.01</v>
       </c>
       <c r="N45">
-        <v>0.78</v>
+        <v>5.59</v>
       </c>
       <c r="Q45" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="R45">
-        <v>0.31</v>
+        <v>5.45</v>
       </c>
       <c r="S45">
-        <v>-1.25</v>
+        <v>6.59</v>
       </c>
       <c r="T45">
-        <v>0.1</v>
+        <v>5.52</v>
       </c>
       <c r="U45">
-        <v>0.51</v>
+        <v>5.01</v>
       </c>
       <c r="V45">
-        <v>-0.3</v>
+        <v>5.47</v>
       </c>
       <c r="Y45" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Z45">
-        <v>4.76</v>
+        <v>5.24</v>
       </c>
       <c r="AA45">
-        <v>2.66</v>
+        <v>6.16</v>
       </c>
       <c r="AB45">
-        <v>4.25</v>
+        <v>5.52</v>
       </c>
       <c r="AC45">
-        <v>4.17</v>
+        <v>5.02</v>
       </c>
       <c r="AD45">
-        <v>3.57</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="46" spans="1:30">
       <c r="A46" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B46">
-        <v>1136</v>
+        <v>2415</v>
       </c>
       <c r="C46">
-        <v>954</v>
+        <v>2784</v>
       </c>
       <c r="D46">
-        <v>1100</v>
+        <v>1727</v>
       </c>
       <c r="E46">
-        <v>1113</v>
+        <v>5541</v>
       </c>
       <c r="F46">
-        <v>907</v>
+        <v>1355</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J46">
-        <v>973</v>
+        <v>2039</v>
       </c>
       <c r="K46">
-        <v>861</v>
+        <v>3327</v>
       </c>
       <c r="L46">
-        <v>948</v>
+        <v>1727</v>
       </c>
       <c r="M46">
-        <v>966</v>
+        <v>5541</v>
       </c>
       <c r="N46">
-        <v>781</v>
+        <v>1355</v>
       </c>
       <c r="Q46" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="R46">
-        <v>877</v>
+        <v>2039</v>
       </c>
       <c r="S46">
-        <v>806</v>
+        <v>3327</v>
       </c>
       <c r="T46">
-        <v>859</v>
+        <v>1339</v>
       </c>
       <c r="U46">
-        <v>872</v>
+        <v>5541</v>
       </c>
       <c r="V46">
-        <v>706</v>
+        <v>2108</v>
       </c>
       <c r="Y46" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="Z46">
-        <v>1226</v>
+        <v>1608</v>
       </c>
       <c r="AA46">
-        <v>1070</v>
+        <v>3229</v>
       </c>
       <c r="AB46">
-        <v>1169</v>
+        <v>1339</v>
       </c>
       <c r="AC46">
-        <v>1114</v>
+        <v>4927</v>
       </c>
       <c r="AD46">
-        <v>970</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="47" spans="1:30">
       <c r="A47" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B47">
+        <v>2.34</v>
+      </c>
+      <c r="C47">
+        <v>0.13</v>
+      </c>
+      <c r="D47">
+        <v>1.8</v>
+      </c>
+      <c r="E47">
+        <v>1.95</v>
+      </c>
+      <c r="F47">
+        <v>1.21</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J47">
+        <v>1.61</v>
+      </c>
+      <c r="K47">
+        <v>-0.42</v>
+      </c>
+      <c r="L47">
+        <v>1.14</v>
+      </c>
+      <c r="M47">
+        <v>1.2</v>
+      </c>
+      <c r="N47">
+        <v>0.55</v>
+      </c>
+      <c r="Q47" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R47">
+        <v>0.59</v>
+      </c>
+      <c r="S47">
+        <v>-1.19</v>
+      </c>
+      <c r="T47">
+        <v>0.19</v>
+      </c>
+      <c r="U47">
+        <v>0.16</v>
+      </c>
+      <c r="V47">
+        <v>-0.37</v>
+      </c>
+      <c r="Y47" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z47">
+        <v>5.34</v>
+      </c>
+      <c r="AA47">
+        <v>2.76</v>
+      </c>
+      <c r="AB47">
+        <v>4.7</v>
+      </c>
+      <c r="AC47">
+        <v>3.77</v>
+      </c>
+      <c r="AD47">
+        <v>3.48</v>
+      </c>
+    </row>
+    <row r="48" spans="1:30">
+      <c r="A48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B48">
+        <v>1.06</v>
+      </c>
+      <c r="C48">
+        <v>-0.11</v>
+      </c>
+      <c r="D48">
+        <v>0.91</v>
+      </c>
+      <c r="E48">
+        <v>1.68</v>
+      </c>
+      <c r="F48">
+        <v>0.97</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J48">
+        <v>0.57</v>
+      </c>
+      <c r="K48">
+        <v>-0.67</v>
+      </c>
+      <c r="L48">
+        <v>0.29</v>
+      </c>
+      <c r="M48">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="N48">
+        <v>0.32</v>
+      </c>
+      <c r="Q48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R48">
+        <v>-0.34</v>
+      </c>
+      <c r="S48">
+        <v>-1.41</v>
+      </c>
+      <c r="T48">
+        <v>-0.43</v>
+      </c>
+      <c r="U48">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="V48">
+        <v>-0.58</v>
+      </c>
+      <c r="Y48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z48">
+        <v>4.02</v>
+      </c>
+      <c r="AA48">
+        <v>2.5</v>
+      </c>
+      <c r="AB48">
+        <v>3.62</v>
+      </c>
+      <c r="AC48">
+        <v>3.5</v>
+      </c>
+      <c r="AD48">
+        <v>3.23</v>
+      </c>
+    </row>
+    <row r="49" spans="1:30">
+      <c r="A49" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B47">
-        <v>1.206</v>
-      </c>
-      <c r="C47">
-        <v>0.336</v>
-      </c>
-      <c r="D47">
-        <v>1.004</v>
-      </c>
-      <c r="E47">
-        <v>0.978</v>
-      </c>
-      <c r="F47">
-        <v>0.6909999999999999</v>
-      </c>
-      <c r="I47" s="2" t="s">
+      <c r="B49">
+        <v>920</v>
+      </c>
+      <c r="C49">
+        <v>880</v>
+      </c>
+      <c r="D49">
+        <v>914</v>
+      </c>
+      <c r="E49">
+        <v>946</v>
+      </c>
+      <c r="F49">
+        <v>786</v>
+      </c>
+      <c r="I49" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J47">
-        <v>0.711</v>
-      </c>
-      <c r="K47">
-        <v>0.052</v>
-      </c>
-      <c r="L47">
-        <v>0.545</v>
-      </c>
-      <c r="M47">
-        <v>0.532</v>
-      </c>
-      <c r="N47">
-        <v>0.309</v>
-      </c>
-      <c r="Q47" s="2" t="s">
+      <c r="J49">
+        <v>875</v>
+      </c>
+      <c r="K49">
+        <v>846</v>
+      </c>
+      <c r="L49">
+        <v>872</v>
+      </c>
+      <c r="M49">
+        <v>898</v>
+      </c>
+      <c r="N49">
+        <v>744</v>
+      </c>
+      <c r="Q49" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="R47">
-        <v>0.423</v>
-      </c>
-      <c r="S47">
-        <v>-0.114</v>
-      </c>
-      <c r="T47">
-        <v>0.277</v>
-      </c>
-      <c r="U47">
-        <v>0.251</v>
-      </c>
-      <c r="V47">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="Y47" s="2" t="s">
+      <c r="R49">
+        <v>806</v>
+      </c>
+      <c r="S49">
+        <v>795</v>
+      </c>
+      <c r="T49">
+        <v>809</v>
+      </c>
+      <c r="U49">
+        <v>828</v>
+      </c>
+      <c r="V49">
+        <v>684</v>
+      </c>
+      <c r="Y49" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Z47">
-        <v>1.475</v>
-      </c>
-      <c r="AA47">
-        <v>0.68</v>
-      </c>
-      <c r="AB47">
-        <v>1.209</v>
-      </c>
-      <c r="AC47">
-        <v>0.982</v>
-      </c>
-      <c r="AD47">
-        <v>0.878</v>
+      <c r="Z49">
+        <v>1121</v>
+      </c>
+      <c r="AA49">
+        <v>1058</v>
+      </c>
+      <c r="AB49">
+        <v>1108</v>
+      </c>
+      <c r="AC49">
+        <v>1067</v>
+      </c>
+      <c r="AD49">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="50" spans="1:30">
+      <c r="A50" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B50">
+        <v>0.5590000000000001</v>
+      </c>
+      <c r="C50">
+        <v>0.116</v>
+      </c>
+      <c r="D50">
+        <v>0.449</v>
+      </c>
+      <c r="E50">
+        <v>0.478</v>
+      </c>
+      <c r="F50">
+        <v>0.33</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J50">
+        <v>0.416</v>
+      </c>
+      <c r="K50">
+        <v>0.006</v>
+      </c>
+      <c r="L50">
+        <v>0.318</v>
+      </c>
+      <c r="M50">
+        <v>0.33</v>
+      </c>
+      <c r="N50">
+        <v>0.199</v>
+      </c>
+      <c r="Q50" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="R50">
+        <v>0.213</v>
+      </c>
+      <c r="S50">
+        <v>-0.147</v>
+      </c>
+      <c r="T50">
+        <v>0.128</v>
+      </c>
+      <c r="U50">
+        <v>0.123</v>
+      </c>
+      <c r="V50">
+        <v>0.017</v>
+      </c>
+      <c r="Y50" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="Z50">
+        <v>1.16</v>
+      </c>
+      <c r="AA50">
+        <v>0.642</v>
+      </c>
+      <c r="AB50">
+        <v>1.027</v>
+      </c>
+      <c r="AC50">
+        <v>0.843</v>
+      </c>
+      <c r="AD50">
+        <v>0.785</v>
       </c>
     </row>
   </sheetData>

</xml_diff>